<commit_message>
chore: 엑셀 임시파일 gitignore 추가
</commit_message>
<xml_diff>
--- a/데이터/opened_course2026_1.xlsx
+++ b/데이터/opened_course2026_1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0d90a49386c3f612/바탕 화면/AI융개_팀플/데이터/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\AI융개_팀플\데이터\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="167" documentId="8_{2611B527-B02A-4874-942C-B92529217652}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{468B97B9-AEA5-442E-8BA2-552C62E8C156}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="심화전공2026_1" sheetId="6" r:id="rId1"/>
@@ -3097,10 +3097,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>